<commit_message>
Add scheduling workflow and approval pipeline
This change adds the new WF05_Schedule_Posts workflow to consume approved content and posting-time configuration for scheduled publishing, while updating the human approval workflow to handle approval emails more robustly. It also refreshes generated UiPath metadata, workbook data files, and related local build artifacts, and removes obsolete image/tooling files from the earlier content-generation setup.
</commit_message>
<xml_diff>
--- a/Config/Config.xlsx
+++ b/Config/Config.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://groupecgi-my.sharepoint.com/personal/ali_mahjoub_cgi_com/Documents/Documents/UiPath/AI Social Media Manager/Config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="8_{04A6FCC9-2EBC-479D-970D-986588D51F89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B629A2F-B48E-48D9-A265-54B66E5280E7}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="8_{04A6FCC9-2EBC-479D-970D-986588D51F89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E404BE14-CE9B-49A8-A987-493D9B6AA468}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{054E92E9-8A22-462D-B45F-2085CB9A574B}"/>
+    <workbookView xWindow="4728" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{054E92E9-8A22-462D-B45F-2085CB9A574B}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="PostingTimes" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -454,6 +455,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB7BAA03-3F80-48E0-B2DA-F05A6A146C2A}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A01977AF-9330-4254-BAF1-FDE769D1C557}">
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -491,7 +501,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">

</xml_diff>